<commit_message>
🔒 [FULL] Daily chip data 2026-05-12 12:39
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-05-11.xlsx
+++ b/data/reports/chip_radar_2026-05-11.xlsx
@@ -1325,7 +1325,7 @@
         <v>7</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" s="3" t="n">
         <v>1613</v>
@@ -1340,9 +1340,9 @@
         <v>2304.43</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" s="5">
+        <v>226</v>
+      </c>
+      <c r="L24" s="6">
         <f>F24*(K24-J24)</f>
         <v/>
       </c>
@@ -1421,7 +1421,7 @@
         <v>5</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G27" s="3" t="n">
         <v>1154</v>
@@ -1436,9 +1436,9 @@
         <v>2309</v>
       </c>
       <c r="K27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" s="5">
+        <v>206</v>
+      </c>
+      <c r="L27" s="6">
         <f>F27*(K27-J27)</f>
         <v/>
       </c>
@@ -1485,7 +1485,7 @@
         <v>2</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29" s="3" t="n">
         <v>1071</v>
@@ -1500,9 +1500,9 @@
         <v>5355</v>
       </c>
       <c r="K29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" s="5">
+        <v>81</v>
+      </c>
+      <c r="L29" s="6">
         <f>F29*(K29-J29)</f>
         <v/>
       </c>
@@ -1549,7 +1549,7 @@
         <v>2</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G31" s="3" t="n">
         <v>787</v>
@@ -1564,9 +1564,9 @@
         <v>3934.5</v>
       </c>
       <c r="K31" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" s="5">
+        <v>48</v>
+      </c>
+      <c r="L31" s="6">
         <f>F31*(K31-J31)</f>
         <v/>
       </c>
@@ -1581,7 +1581,7 @@
         <v>3</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="3" t="n">
         <v>780</v>
@@ -1596,9 +1596,9 @@
         <v>2601.67</v>
       </c>
       <c r="K32" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" s="5">
+        <v>26</v>
+      </c>
+      <c r="L32" s="6">
         <f>F32*(K32-J32)</f>
         <v/>
       </c>
@@ -2979,7 +2979,7 @@
         <v>124</v>
       </c>
       <c r="F71" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G71" s="3" t="n">
         <v>33108</v>
@@ -2994,9 +2994,9 @@
         <v>2670</v>
       </c>
       <c r="K71" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L71" s="5">
+        <v>48</v>
+      </c>
+      <c r="L71" s="6">
         <f>F71*(K71-J71)</f>
         <v/>
       </c>
@@ -3891,7 +3891,7 @@
         <v>3</v>
       </c>
       <c r="F97" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G97" s="3" t="n">
         <v>1633</v>
@@ -3906,9 +3906,9 @@
         <v>5443.67</v>
       </c>
       <c r="K97" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L97" s="5">
+        <v>133</v>
+      </c>
+      <c r="L97" s="6">
         <f>F97*(K97-J97)</f>
         <v/>
       </c>
@@ -6482,7 +6482,7 @@
         <v>124</v>
       </c>
       <c r="F170" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G170" s="3" t="n">
         <v>33108</v>
@@ -6497,9 +6497,9 @@
         <v>2670</v>
       </c>
       <c r="K170" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L170" s="5">
+        <v>48</v>
+      </c>
+      <c r="L170" s="6">
         <f>F170*(K170-J170)</f>
         <v/>
       </c>
@@ -7256,7 +7256,7 @@
         <v>10</v>
       </c>
       <c r="F192" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G192" s="3" t="n">
         <v>6393</v>
@@ -7271,9 +7271,9 @@
         <v>6392.9</v>
       </c>
       <c r="K192" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L192" s="5">
+        <v>18</v>
+      </c>
+      <c r="L192" s="6">
         <f>F192*(K192-J192)</f>
         <v/>
       </c>
@@ -8072,7 +8072,7 @@
         <v>62</v>
       </c>
       <c r="F215" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G215" s="3" t="n">
         <v>13976</v>
@@ -8087,9 +8087,9 @@
         <v>2254.11</v>
       </c>
       <c r="K215" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L215" s="5">
+        <v>740</v>
+      </c>
+      <c r="L215" s="6">
         <f>F215*(K215-J215)</f>
         <v/>
       </c>
@@ -8619,7 +8619,7 @@
         <v>97</v>
       </c>
       <c r="F231" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G231" s="3" t="n">
         <v>2509</v>
@@ -8634,9 +8634,9 @@
         <v>258.66</v>
       </c>
       <c r="K231" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L231" s="5">
+        <v>10</v>
+      </c>
+      <c r="L231" s="6">
         <f>F231*(K231-J231)</f>
         <v/>
       </c>
@@ -8814,7 +8814,7 @@
         <v>10</v>
       </c>
       <c r="F236" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G236" s="3" t="n">
         <v>2826</v>
@@ -8829,9 +8829,9 @@
         <v>2826.4</v>
       </c>
       <c r="K236" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L236" s="5">
+        <v>463</v>
+      </c>
+      <c r="L236" s="6">
         <f>F236*(K236-J236)</f>
         <v/>
       </c>
@@ -11294,7 +11294,7 @@
         <v>3</v>
       </c>
       <c r="F306" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G306" s="3" t="n">
         <v>1633</v>
@@ -11309,9 +11309,9 @@
         <v>5443.67</v>
       </c>
       <c r="K306" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L306" s="5">
+        <v>133</v>
+      </c>
+      <c r="L306" s="6">
         <f>F306*(K306-J306)</f>
         <v/>
       </c>
@@ -13402,7 +13402,7 @@
         <v>38</v>
       </c>
       <c r="F365" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G365" s="3" t="n">
         <v>10121</v>
@@ -13417,9 +13417,9 @@
         <v>2663.47</v>
       </c>
       <c r="K365" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L365" s="5">
+        <v>1191</v>
+      </c>
+      <c r="L365" s="6">
         <f>F365*(K365-J365)</f>
         <v/>
       </c>
@@ -14826,7 +14826,7 @@
         </is>
       </c>
       <c r="E406" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F406" s="3" t="n">
         <v>3</v>
@@ -14841,7 +14841,7 @@
         <v>-1110</v>
       </c>
       <c r="J406" s="4" t="n">
-        <v>0</v>
+        <v>1303</v>
       </c>
       <c r="K406" s="4" t="n">
         <v>4135</v>
@@ -15155,29 +15155,29 @@
     <row r="415" ht="16.5" customHeight="1">
       <c r="D415" s="2" t="inlineStr">
         <is>
-          <t>陽程(3498)</t>
+          <t>蔚華科(3055)</t>
         </is>
       </c>
       <c r="E415" s="3" t="n">
-        <v>887</v>
+        <v>1010</v>
       </c>
       <c r="F415" s="3" t="n">
-        <v>0</v>
+        <v>504</v>
       </c>
       <c r="G415" s="3" t="n">
-        <v>9092</v>
+        <v>10100</v>
       </c>
       <c r="H415" s="3" t="n">
-        <v>0</v>
+        <v>5040</v>
       </c>
       <c r="I415" s="3" t="n">
-        <v>9092</v>
+        <v>5060</v>
       </c>
       <c r="J415" s="4" t="n">
-        <v>102.5</v>
+        <v>100</v>
       </c>
       <c r="K415" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="L415" s="5">
         <f>F415*(K415-J415)</f>
@@ -15187,31 +15187,31 @@
     <row r="416" ht="16.5" customHeight="1">
       <c r="D416" s="2" t="inlineStr">
         <is>
-          <t>正淩(8147)</t>
+          <t>陽程(3498)</t>
         </is>
       </c>
       <c r="E416" s="3" t="n">
-        <v>493</v>
+        <v>887</v>
       </c>
       <c r="F416" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G416" s="3" t="n">
-        <v>8356</v>
+        <v>9092</v>
       </c>
       <c r="H416" s="3" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="I416" s="3" t="n">
-        <v>8324</v>
+        <v>9092</v>
       </c>
       <c r="J416" s="4" t="n">
-        <v>169.5</v>
+        <v>102.5</v>
       </c>
       <c r="K416" s="4" t="n">
-        <v>160</v>
-      </c>
-      <c r="L416" s="6">
+        <v>0</v>
+      </c>
+      <c r="L416" s="5">
         <f>F416*(K416-J416)</f>
         <v/>
       </c>
@@ -15219,31 +15219,31 @@
     <row r="417" ht="16.5" customHeight="1">
       <c r="D417" s="2" t="inlineStr">
         <is>
-          <t>群聯(8299)</t>
+          <t>正淩(8147)</t>
         </is>
       </c>
       <c r="E417" s="3" t="n">
-        <v>26</v>
+        <v>493</v>
       </c>
       <c r="F417" s="3" t="n">
         <v>2</v>
       </c>
       <c r="G417" s="3" t="n">
-        <v>6994</v>
+        <v>8356</v>
       </c>
       <c r="H417" s="3" t="n">
-        <v>642</v>
+        <v>32</v>
       </c>
       <c r="I417" s="3" t="n">
-        <v>6352</v>
+        <v>8324</v>
       </c>
       <c r="J417" s="4" t="n">
-        <v>2689.92</v>
+        <v>169.5</v>
       </c>
       <c r="K417" s="4" t="n">
-        <v>3210.5</v>
-      </c>
-      <c r="L417" s="5">
+        <v>160</v>
+      </c>
+      <c r="L417" s="6">
         <f>F417*(K417-J417)</f>
         <v/>
       </c>
@@ -15251,31 +15251,31 @@
     <row r="418" ht="16.5" customHeight="1">
       <c r="D418" s="2" t="inlineStr">
         <is>
-          <t>強茂(2481)</t>
+          <t>群聯(8299)</t>
         </is>
       </c>
       <c r="E418" s="3" t="n">
-        <v>508</v>
+        <v>26</v>
       </c>
       <c r="F418" s="3" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="G418" s="3" t="n">
-        <v>5533</v>
+        <v>6994</v>
       </c>
       <c r="H418" s="3" t="n">
-        <v>238</v>
+        <v>642</v>
       </c>
       <c r="I418" s="3" t="n">
-        <v>5295</v>
+        <v>6352</v>
       </c>
       <c r="J418" s="4" t="n">
-        <v>108.91</v>
+        <v>2689.92</v>
       </c>
       <c r="K418" s="4" t="n">
-        <v>108.09</v>
-      </c>
-      <c r="L418" s="6">
+        <v>3210.5</v>
+      </c>
+      <c r="L418" s="5">
         <f>F418*(K418-J418)</f>
         <v/>
       </c>
@@ -15421,7 +15421,7 @@
         <v>5</v>
       </c>
       <c r="F422" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G422" s="3" t="n">
         <v>2663</v>
@@ -15436,9 +15436,9 @@
         <v>5326</v>
       </c>
       <c r="K422" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L422" s="5">
+        <v>672</v>
+      </c>
+      <c r="L422" s="6">
         <f>F422*(K422-J422)</f>
         <v/>
       </c>
@@ -16407,7 +16407,7 @@
         <v>4</v>
       </c>
       <c r="F450" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G450" s="3" t="n">
         <v>1650</v>
@@ -16422,9 +16422,9 @@
         <v>4126.25</v>
       </c>
       <c r="K450" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L450" s="5">
+        <v>1672</v>
+      </c>
+      <c r="L450" s="6">
         <f>F450*(K450-J450)</f>
         <v/>
       </c>

</xml_diff>